<commit_message>
filled table and added evidences
</commit_message>
<xml_diff>
--- a/Teste_de_sistemas/Trabalhos/ATIVIDADE_TESTES_EXPLORATORIOS_VITOR_RAZIA_BUBOLS/02_matriz_de_testes/Matriz_de_testes.xlsx
+++ b/Teste_de_sistemas/Trabalhos/ATIVIDADE_TESTES_EXPLORATORIOS_VITOR_RAZIA_BUBOLS/02_matriz_de_testes/Matriz_de_testes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vitor_bubols\SENAI_FASE3\Teste_de_sistemas\Trabalhos\ATIVIDADE_TESTES_EXPLORATORIOS_VITOR_RAZIA_BUBOLS\02_matriz_de_testes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A00817C-0644-4BF5-A6F1-3AAECC88719B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E97C5AEB-7E1D-4079-8C34-98AC69C1F0DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="80">
   <si>
     <t>SUITE</t>
   </si>
@@ -60,63 +60,30 @@
     <t>Login com campos vazios</t>
   </si>
   <si>
-    <t>Navegação</t>
-  </si>
-  <si>
-    <t>NAV-004</t>
-  </si>
-  <si>
-    <t>Navegar entre páginas do painel</t>
-  </si>
-  <si>
     <t>Rooms</t>
   </si>
   <si>
-    <t>ROOM-005</t>
-  </si>
-  <si>
     <t>Visualizar lista de quartos</t>
   </si>
   <si>
-    <t>ROOM-006</t>
-  </si>
-  <si>
     <t>Criar novo quarto</t>
   </si>
   <si>
-    <t>ROOM-007</t>
-  </si>
-  <si>
     <t>Criar quarto com dados inválidos</t>
   </si>
   <si>
     <t>Booking</t>
   </si>
   <si>
-    <t>BOOK-008</t>
-  </si>
-  <si>
     <t>Visualizar reservas existentes</t>
   </si>
   <si>
     <t>Messages</t>
   </si>
   <si>
-    <t>MSG-009</t>
-  </si>
-  <si>
     <t>Visualizar mensagens recebidas</t>
   </si>
   <si>
-    <t>Usabilidade</t>
-  </si>
-  <si>
-    <t>UI-010</t>
-  </si>
-  <si>
-    <t>Verificar feedback visual após ações</t>
-  </si>
-  <si>
     <t>Funcionalidade</t>
   </si>
   <si>
@@ -133,9 +100,6 @@
   </si>
   <si>
     <t>Tipo</t>
-  </si>
-  <si>
-    <t>Tela recarrega sem mensagem</t>
   </si>
   <si>
     <t>Exploratório</t>
@@ -163,6 +127,185 @@
   </si>
   <si>
     <t>N/A</t>
+  </si>
+  <si>
+    <t>ROOM-001</t>
+  </si>
+  <si>
+    <t>ROOM-002</t>
+  </si>
+  <si>
+    <t>ROOM-003</t>
+  </si>
+  <si>
+    <t>BOOK-001</t>
+  </si>
+  <si>
+    <t>MSG-001</t>
+  </si>
+  <si>
+    <t>UI-001</t>
+  </si>
+  <si>
+    <t>Sistema realiza o login normalmente</t>
+  </si>
+  <si>
+    <t>Evidência</t>
+  </si>
+  <si>
+    <t>EVID_LOGIN_LOGIN-001, EVID_LOGIN_LOGIN-001_response</t>
+  </si>
+  <si>
+    <t>Sistema notifica que credencias são invalidas</t>
+  </si>
+  <si>
+    <t>EVID_LOGIN_LOGIN-002</t>
+  </si>
+  <si>
+    <t>Sistema notifica que credencias são invalidas mas não que estão vazias</t>
+  </si>
+  <si>
+    <t>Leve</t>
+  </si>
+  <si>
+    <t>EVID_LOGIN_LOGIN-003</t>
+  </si>
+  <si>
+    <t>1. Acessar o site
+2. Inserir credenciais validas
+3. Logar na plataforma
+4. Ir na aba de "Rooms"</t>
+  </si>
+  <si>
+    <t>Sistema deve apresentar a lista de quartos</t>
+  </si>
+  <si>
+    <t>Sistema apresenta a lista de quartos normalmente</t>
+  </si>
+  <si>
+    <t>EVID_ROOMS_ROOM_001</t>
+  </si>
+  <si>
+    <t>1. Acessar o site
+2. Inserir credenciais validas
+3. Logar na plataforma
+4. Ir na aba de "Rooms"
+5. Preencher informações
+6. Criar novo quarto</t>
+  </si>
+  <si>
+    <t>Sistema deve criar o novo quarto baseado nas informações preenchidas</t>
+  </si>
+  <si>
+    <t>1. Acessar o site
+2. Inserir credenciais validas
+3. Logar na plataforma
+4. Ir na aba de "Rooms"
+5. Preencher informações com dados inválidos
+6. Tentar criar novo quarto</t>
+  </si>
+  <si>
+    <t>Sistema deve notificar informarções inválidas e não criar o quarto</t>
+  </si>
+  <si>
+    <t>Sistema criou o novo quarto baseado nas informações preenchidas</t>
+  </si>
+  <si>
+    <t>Sistema notificou a informação inválida e não criou o novo quarto</t>
+  </si>
+  <si>
+    <t>EVID_ROOMS_ROOM_002</t>
+  </si>
+  <si>
+    <t>EVID_ROOMS_ROOM_003</t>
+  </si>
+  <si>
+    <t>Book</t>
+  </si>
+  <si>
+    <t>1. Acessar o site
+2. Inserir credenciais validas
+3. Logar na plataforma
+4. Ir na aba de "Report"
+5. Visualizar no calendário as reservas feitas</t>
+  </si>
+  <si>
+    <t>Sistema deve mostrar de forma clara a reserva feita por quem, qual quarto e data</t>
+  </si>
+  <si>
+    <t>Sistema mostra no calendário o nome de quem reservou, o quarto e a data</t>
+  </si>
+  <si>
+    <t>EVID_BOOKING_BOOK-001</t>
+  </si>
+  <si>
+    <t>1. Acessar o site
+2. Inserir credenciais validas
+3. Logar na plataforma
+4. Ir na aba de "Messages"
+5. Visualizar as mensagens</t>
+  </si>
+  <si>
+    <t>O sistema deve mostrar de forma a clara as mensagens recebidas</t>
+  </si>
+  <si>
+    <t>O sistema mostra de forma clara as mensagens recebidas, após clicar nelas abre uma nova janela com mais informações da mensagem</t>
+  </si>
+  <si>
+    <t>EVID_MESSAGES_MSG-001_list, EVID_MESSAGES_MSG-001_message</t>
+  </si>
+  <si>
+    <t>Verificar responsividade da página</t>
+  </si>
+  <si>
+    <t>User Interface</t>
+  </si>
+  <si>
+    <t>1. Acessar o site
+2. Inserir credenciais validas
+3. Logar na plataforma
+4. Abrir o devTools no navegador
+5. Testar resoluções diferentes ao navegar pelas páginas</t>
+  </si>
+  <si>
+    <t>O sistema deve continuar responsivo, sem apresentar componentes quebrados e todas funcionalidades operando normalmente</t>
+  </si>
+  <si>
+    <t>Performance</t>
+  </si>
+  <si>
+    <t>PERF-001</t>
+  </si>
+  <si>
+    <t>Avaliar tempo de carregamento das páginas</t>
+  </si>
+  <si>
+    <t>1. Acessar o site
+2. Inserir credenciais válidas
+3. Realizar login na plataforma
+4. Abrir o DevTools do navegador (F12)
+5. Acessar a aba "Network"
+6. Navegar entre as páginas (Rooms, Bookings, Messages)
+7. Observar o tempo de carregamento das requisições
+8. Repetir o processo para validar consistência dos tempos</t>
+  </si>
+  <si>
+    <t>As páginas devem carregar em tempo aceitável, sem atrasos excessivos ou falhas no carregamento dos recursos.</t>
+  </si>
+  <si>
+    <t>Interface</t>
+  </si>
+  <si>
+    <t>O sistema continua responsivo, nenhum componente quebra e todas funcionalidades continuam operando normalmente</t>
+  </si>
+  <si>
+    <t>EVID_INTERFACE_UI-001_1080x732, EVID_INTERFACE_UI-001_414x896, EVID_INTERFACE_UI-001_344x882</t>
+  </si>
+  <si>
+    <t>As páginas carregam rápido e ao navegar entre elas várias vezes já guardam as informações no cache, tornando ainda menoro tempo de carregamento</t>
+  </si>
+  <si>
+    <t>EVID_PERFORMANCE_PERF-001_ROOMS, EVID_PERFORMANCE_PERF-001_REPORT, EVID_PERFORMANCE_PERF-001_MESSAGES, EVID_PERFORMANCE_PERF-001_BRANDING</t>
   </si>
 </sst>
 </file>
@@ -248,7 +391,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -274,7 +417,6 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -291,7 +433,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -584,12 +726,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="33.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="33" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="24.7109375" bestFit="1" customWidth="1"/>
@@ -598,7 +740,7 @@
     <col min="9" max="9" width="11.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -609,25 +751,28 @@
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>34</v>
+        <v>23</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="75" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>3</v>
       </c>
@@ -640,23 +785,26 @@
       <c r="D2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="10" t="s">
+      <c r="E2" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="G2" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="F2" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="G2" s="10" t="s">
-        <v>35</v>
-      </c>
       <c r="H2" s="3" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>36</v>
+        <v>24</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>39</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="75" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>3</v>
       </c>
@@ -669,17 +817,26 @@
       <c r="D3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="F3" s="10" t="s">
+      <c r="E3" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="G3" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J3" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="G3" s="10"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
     </row>
-    <row r="4" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
@@ -692,136 +849,250 @@
       <c r="D4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="F4" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="G4" s="10"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
+      <c r="E4" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="G4" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>44</v>
+      </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="G5" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="90" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="F6" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="G6" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="105" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="D7" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="G7" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="90" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="B8" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="4"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
+      <c r="D8" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="G8" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="J8" s="5" t="s">
+        <v>61</v>
+      </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6" s="4" t="s">
+    <row r="9" spans="1:10" ht="75" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="B9" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="4"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="11"/>
-      <c r="H6" s="4"/>
-      <c r="I6" s="4"/>
+      <c r="D9" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E9" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="G9" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>65</v>
+      </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D7" s="4"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
+    <row r="10" spans="1:10" ht="90" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="E10" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="F10" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="G10" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="J10" s="7" t="s">
+        <v>77</v>
+      </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D8" s="5"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12"/>
-      <c r="H8" s="5"/>
-      <c r="I8" s="5"/>
+    <row r="11" spans="1:10" ht="180" x14ac:dyDescent="0.25">
+      <c r="A11" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="E11" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="F11" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="G11" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="H11" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="I11" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>79</v>
+      </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="D9" s="6"/>
-      <c r="E9" s="13"/>
-      <c r="F9" s="13"/>
-      <c r="G9" s="13"/>
-      <c r="H9" s="6"/>
-      <c r="I9" s="6"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="D10" s="7"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="14"/>
-      <c r="H10" s="7"/>
-      <c r="I10" s="7"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D11" s="9"/>
-      <c r="E11" s="15"/>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
-      <c r="H11" s="9"/>
-      <c r="I11" s="9"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>

</xml_diff>